<commit_message>
format colors in Excel template
</commit_message>
<xml_diff>
--- a/api/templates/device_calibration_report/en.xlsx
+++ b/api/templates/device_calibration_report/en.xlsx
@@ -182,7 +182,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -195,6 +195,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -243,7 +246,54 @@
     <cellStyle name="Hyperlink" xfId="41" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="8">
+    <dxf>
+      <fill>
+        <gradientFill type="path" left="0.5" right="0.5" top="0.5" bottom="0.5">
+          <stop position="0">
+            <color theme="0"/>
+          </stop>
+          <stop position="1">
+            <color rgb="FFFF0000"/>
+          </stop>
+        </gradientFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -269,10 +319,16 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4">
     <tableStyle name="MySqlDefault" pivot="0" table="0" count="2">
-      <tableStyleElement type="wholeTable" dxfId="1"/>
-      <tableStyleElement type="headerRow" dxfId="0"/>
+      <tableStyleElement type="wholeTable" dxfId="7"/>
+      <tableStyleElement type="headerRow" dxfId="6"/>
     </tableStyle>
   </tableStyles>
+  <colors>
+    <mruColors>
+      <color rgb="FFFFC7CE"/>
+      <color rgb="FFFF7C80"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -664,7 +720,7 @@
       <c r="B7" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="8" t="s">
         <v>11</v>
       </c>
       <c r="D7" s="7" t="s">
@@ -672,6 +728,17 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="C7:C999999">
+    <cfRule type="cellIs" dxfId="5" priority="2" stopIfTrue="1" operator="greaterThan">
+      <formula>DATE(YEAR(TODAY())-1, MONTH(TODAY()), DAY(TODAY()))</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="1" stopIfTrue="1" operator="greaterThan">
+      <formula>DATE(YEAR(TODAY()), MONTH(TODAY())-8, DAY(TODAY()))</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="3" stopIfTrue="1" operator="greaterThan">
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>